<commit_message>
Planilla por empresa: catálogo de empresas y periodos por empresa y mes
</commit_message>
<xml_diff>
--- a/Rutas de Viajes.xlsx
+++ b/Rutas de Viajes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8f0925b7c2ae613a/Escritorio/erp transport/erp-transporte/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FA786C9E-8C24-4BBC-B531-F2C7D4FAA509}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{FA786C9E-8C24-4BBC-B531-F2C7D4FAA509}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{886A8074-55B9-44B7-BA1F-EC17FBCB594F}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="139">
   <si>
     <t>RUTA</t>
   </si>
@@ -276,9 +276,6 @@
   </si>
   <si>
     <t>Pucallpa-Chanchamayo-Lima.Pucallpa</t>
-  </si>
-  <si>
-    <t>800 io 900</t>
   </si>
   <si>
     <t>Pucallpa</t>
@@ -970,13 +967,13 @@
         <v>400</v>
       </c>
       <c r="F2" t="s">
+        <v>80</v>
+      </c>
+      <c r="G2" t="s">
         <v>81</v>
       </c>
-      <c r="G2" t="s">
-        <v>82</v>
-      </c>
       <c r="H2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.4">
@@ -987,10 +984,10 @@
         <v>200</v>
       </c>
       <c r="F3" t="s">
+        <v>80</v>
+      </c>
+      <c r="G3" t="s">
         <v>81</v>
-      </c>
-      <c r="G3" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.4">
@@ -1001,10 +998,10 @@
         <v>200</v>
       </c>
       <c r="F4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.4">
@@ -1015,13 +1012,13 @@
         <v>486</v>
       </c>
       <c r="F5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.4">
@@ -1032,13 +1029,13 @@
         <v>486</v>
       </c>
       <c r="F6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.4">
@@ -1049,13 +1046,13 @@
         <v>345</v>
       </c>
       <c r="F7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.4">
@@ -1066,13 +1063,13 @@
         <v>450</v>
       </c>
       <c r="F8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.4">
@@ -1083,13 +1080,13 @@
         <v>620</v>
       </c>
       <c r="F9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.4">
@@ -1100,13 +1097,13 @@
         <v>620</v>
       </c>
       <c r="F10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G10" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.4">
@@ -1117,13 +1114,13 @@
         <v>720</v>
       </c>
       <c r="F11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.4">
@@ -1134,13 +1131,13 @@
         <v>320</v>
       </c>
       <c r="F12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G12" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.4">
@@ -1151,13 +1148,13 @@
         <v>720</v>
       </c>
       <c r="F13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.4">
@@ -1168,13 +1165,13 @@
         <v>810</v>
       </c>
       <c r="F14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G14" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.4">
@@ -1185,13 +1182,13 @@
         <v>540</v>
       </c>
       <c r="F15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G15" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.4">
@@ -1202,13 +1199,13 @@
         <v>320</v>
       </c>
       <c r="F16" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G16" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H16" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.4">
@@ -1219,13 +1216,13 @@
         <v>600</v>
       </c>
       <c r="F17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.4">
@@ -1236,13 +1233,13 @@
         <v>180</v>
       </c>
       <c r="F18" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G18" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H18" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.4">
@@ -1253,13 +1250,13 @@
         <v>80</v>
       </c>
       <c r="F19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G19" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.4">
@@ -1270,13 +1267,13 @@
         <v>200</v>
       </c>
       <c r="F20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G20" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.4">
@@ -1285,13 +1282,13 @@
       </c>
       <c r="B21" s="2"/>
       <c r="F21" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G21" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H21" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.4">
@@ -1300,13 +1297,13 @@
       </c>
       <c r="B22" s="2"/>
       <c r="F22" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G22" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H22" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.4">
@@ -1317,30 +1314,30 @@
         <v>500</v>
       </c>
       <c r="F23" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G23" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H23" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="5" t="s">
-        <v>80</v>
+      <c r="B24" s="5">
+        <v>800</v>
       </c>
       <c r="F24" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G24" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H24" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.4">
@@ -1351,13 +1348,13 @@
         <v>1100</v>
       </c>
       <c r="F25" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G25" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H25" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.4">
@@ -1368,13 +1365,13 @@
         <v>900</v>
       </c>
       <c r="F26" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G26" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H26" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.4">
@@ -1385,13 +1382,13 @@
         <v>900</v>
       </c>
       <c r="F27" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G27" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H27" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.4">
@@ -1402,13 +1399,13 @@
         <v>750</v>
       </c>
       <c r="F28" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G28" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H28" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.4">
@@ -1419,13 +1416,13 @@
         <v>500</v>
       </c>
       <c r="F29" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G29" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H29" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.4">
@@ -1436,13 +1433,13 @@
         <v>375</v>
       </c>
       <c r="F30" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G30" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H30" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.4">
@@ -1451,16 +1448,16 @@
       </c>
       <c r="B31" s="2"/>
       <c r="F31" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G31" t="s">
+        <v>104</v>
+      </c>
+      <c r="H31" t="s">
         <v>105</v>
       </c>
-      <c r="H31" t="s">
-        <v>106</v>
-      </c>
       <c r="I31" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.4">
@@ -1471,19 +1468,19 @@
         <v>1100</v>
       </c>
       <c r="F32" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G32" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H32" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I32" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J32" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.4">
@@ -1494,13 +1491,13 @@
         <v>220</v>
       </c>
       <c r="F33" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G33" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H33" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.4">
@@ -1511,13 +1508,13 @@
         <v>910</v>
       </c>
       <c r="F34" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G34" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H34" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.4">
@@ -1528,13 +1525,13 @@
         <v>750</v>
       </c>
       <c r="F35" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G35" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H35" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.4">
@@ -1545,13 +1542,13 @@
         <v>240</v>
       </c>
       <c r="F36" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G36" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H36" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.4">
@@ -1560,13 +1557,13 @@
       </c>
       <c r="B37" s="2"/>
       <c r="F37" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G37" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H37" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.4">
@@ -1577,13 +1574,13 @@
         <v>140</v>
       </c>
       <c r="F38" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G38" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H38" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.4">
@@ -1594,13 +1591,13 @@
         <v>140</v>
       </c>
       <c r="F39" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G39" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H39" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.4">
@@ -1611,10 +1608,10 @@
         <v>80</v>
       </c>
       <c r="F40" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G40" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.4">
@@ -1625,13 +1622,13 @@
         <v>400</v>
       </c>
       <c r="F41" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G41" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H41" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.4">
@@ -1642,13 +1639,13 @@
         <v>600</v>
       </c>
       <c r="F42" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G42" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H42" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.4">
@@ -1659,13 +1656,13 @@
         <v>650</v>
       </c>
       <c r="F43" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G43" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H43" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.4">
@@ -1676,16 +1673,16 @@
         <v>600</v>
       </c>
       <c r="F44" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G44" t="s">
+        <v>116</v>
+      </c>
+      <c r="H44" t="s">
         <v>117</v>
       </c>
-      <c r="H44" t="s">
-        <v>118</v>
-      </c>
       <c r="I44" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.4">
@@ -1696,13 +1693,13 @@
         <v>250</v>
       </c>
       <c r="F45" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G45" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H45" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.4">
@@ -1713,13 +1710,13 @@
         <v>220</v>
       </c>
       <c r="F46" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G46" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H46" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.4">
@@ -1730,13 +1727,13 @@
         <v>220</v>
       </c>
       <c r="F47" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G47" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H47" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.4">
@@ -1747,13 +1744,13 @@
         <v>180</v>
       </c>
       <c r="F48" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G48" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H48" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.4">
@@ -1764,13 +1761,13 @@
         <v>400</v>
       </c>
       <c r="F49" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G49" t="s">
+        <v>80</v>
+      </c>
+      <c r="H49" t="s">
         <v>81</v>
-      </c>
-      <c r="H49" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.4">
@@ -1781,19 +1778,19 @@
         <v>840</v>
       </c>
       <c r="F50" t="s">
+        <v>119</v>
+      </c>
+      <c r="G50" t="s">
         <v>120</v>
       </c>
-      <c r="G50" t="s">
+      <c r="H50" t="s">
         <v>121</v>
       </c>
-      <c r="H50" t="s">
-        <v>122</v>
-      </c>
       <c r="I50" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="J50" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.4">
@@ -1804,13 +1801,13 @@
         <v>220</v>
       </c>
       <c r="F51" t="s">
+        <v>82</v>
+      </c>
+      <c r="G51" t="s">
         <v>83</v>
       </c>
-      <c r="G51" t="s">
-        <v>84</v>
-      </c>
       <c r="H51" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.4">
@@ -1821,16 +1818,16 @@
         <v>800</v>
       </c>
       <c r="F52" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G52" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H52" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I52" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.4">
@@ -1841,13 +1838,13 @@
         <v>500</v>
       </c>
       <c r="F53" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G53" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H53" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.4">
@@ -1856,13 +1853,13 @@
       </c>
       <c r="B54" s="2"/>
       <c r="F54" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G54" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H54" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.4">
@@ -1873,13 +1870,13 @@
         <v>500</v>
       </c>
       <c r="F55" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G55" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H55" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.4">
@@ -1890,13 +1887,13 @@
         <v>250</v>
       </c>
       <c r="F56" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G56" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H56" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.4">
@@ -1907,13 +1904,13 @@
         <v>600</v>
       </c>
       <c r="F57" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G57" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H57" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.4">
@@ -1924,13 +1921,13 @@
         <v>386</v>
       </c>
       <c r="F58" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G58" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H58" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.4">
@@ -1941,13 +1938,13 @@
         <v>190</v>
       </c>
       <c r="F59" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G59" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="H59" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.4">
@@ -1958,13 +1955,13 @@
         <v>370</v>
       </c>
       <c r="F60" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G60" t="s">
+        <v>126</v>
+      </c>
+      <c r="H60" t="s">
         <v>127</v>
-      </c>
-      <c r="H60" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.4">
@@ -1975,13 +1972,13 @@
         <v>516</v>
       </c>
       <c r="F61" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G61" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H61" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.4">
@@ -1992,13 +1989,13 @@
         <v>600</v>
       </c>
       <c r="F62" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G62" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H62" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.4">
@@ -2009,10 +2006,10 @@
         <v>300</v>
       </c>
       <c r="F63" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G63" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.4">
@@ -2023,10 +2020,10 @@
         <v>300</v>
       </c>
       <c r="F64" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G64" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.4">
@@ -2037,13 +2034,13 @@
         <v>750</v>
       </c>
       <c r="F65" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G65" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H65" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.4">
@@ -2054,13 +2051,13 @@
         <v>650</v>
       </c>
       <c r="F66" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G66" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H66" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.4">
@@ -2071,13 +2068,13 @@
         <v>500</v>
       </c>
       <c r="F67" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G67" t="s">
+        <v>130</v>
+      </c>
+      <c r="H67" t="s">
         <v>131</v>
-      </c>
-      <c r="H67" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.4">
@@ -2088,13 +2085,13 @@
         <v>400</v>
       </c>
       <c r="F68" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G68" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H68" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.4">
@@ -2105,13 +2102,13 @@
         <v>700</v>
       </c>
       <c r="F69" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G69" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H69" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.4">
@@ -2122,13 +2119,13 @@
         <v>950</v>
       </c>
       <c r="F70" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G70" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H70" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.4">
@@ -2139,16 +2136,16 @@
         <v>800</v>
       </c>
       <c r="F71" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G71" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H71" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I71" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.4">
@@ -2159,16 +2156,16 @@
         <v>1200</v>
       </c>
       <c r="F72" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G72" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H72" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I72" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.4">
@@ -2179,13 +2176,13 @@
         <v>325</v>
       </c>
       <c r="F73" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G73" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H73" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.4">
@@ -2196,13 +2193,13 @@
         <v>600</v>
       </c>
       <c r="F74" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G74" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H74" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.4">
@@ -2213,13 +2210,13 @@
         <v>750</v>
       </c>
       <c r="F75" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G75" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H75" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.4">
@@ -2230,13 +2227,13 @@
         <v>550</v>
       </c>
       <c r="F76" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G76" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H76" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.4">
@@ -2247,13 +2244,13 @@
         <v>350</v>
       </c>
       <c r="F77" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G77" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H77" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.4">
@@ -2264,16 +2261,16 @@
         <v>710</v>
       </c>
       <c r="F78" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G78" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H78" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I78" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.4">
@@ -2284,19 +2281,19 @@
         <v>800</v>
       </c>
       <c r="F79" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G79" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H79" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I79" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J79" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="80" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.45">
@@ -2307,13 +2304,13 @@
         <v>680</v>
       </c>
       <c r="F80" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G80" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H80" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>

</xml_diff>